<commit_message>
Cleaned up the run file
</commit_message>
<xml_diff>
--- a/WorkBot/refactor-experimental/data/orders/BJ's/BJ's_Bakery_20251109.xlsx
+++ b/WorkBot/refactor-experimental/data/orders/BJ's/BJ's_Bakery_20251109.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,29 @@
       <c r="E2" t="inlineStr">
         <is>
           <t>203.94</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Celsius - Vibe Peach, Tropical, Arctic</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>28.49</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>170.94</t>
         </is>
       </c>
     </row>

</xml_diff>